<commit_message>
Average, minimum and maximum in experiment data sheet
</commit_message>
<xml_diff>
--- a/experiments/data.xlsx
+++ b/experiments/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_Prog\dnn-hyperproperties\experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDCB2BFF-05F1-4EEE-9EEB-FCBA7CDA9D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F9FB1E-4672-4E79-8C44-16EC8F2A6516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B183E387-CFB8-42E0-B1BD-7A71133FCB77}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>#neurons</t>
   </si>
@@ -54,6 +54,15 @@
   </si>
   <si>
     <t>time 5</t>
+  </si>
+  <si>
+    <t>avg</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
   </si>
 </sst>
 </file>
@@ -425,10 +434,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47FF0182-8E1C-4461-94C8-C826B1D71C11}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -447,8 +456,17 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -467,8 +485,20 @@
       <c r="F2">
         <v>3.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2">
+        <f>AVERAGE(B2:F2)</f>
+        <v>2.1999999999999997E-3</v>
+      </c>
+      <c r="H2">
+        <f>MIN(B2:F2)</f>
+        <v>1E-3</v>
+      </c>
+      <c r="I2">
+        <f>MAX(B2:F2)</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -487,8 +517,20 @@
       <c r="F3">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G3">
+        <f t="shared" ref="G3:G10" si="0">AVERAGE(B3:F3)</f>
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H10" si="1">MIN(B3:F3)</f>
+        <v>0.01</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I10" si="2">MAX(B3:F3)</f>
+        <v>1.2E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -507,8 +549,20 @@
       <c r="F4">
         <v>3.9E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>4.0600000000000004E-2</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="1"/>
+        <v>3.9E-2</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="2"/>
+        <v>4.2000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -527,8 +581,20 @@
       <c r="F5">
         <v>0.22800000000000001</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>0.23139999999999999</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="1"/>
+        <v>0.22800000000000001</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="2"/>
+        <v>0.23699999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -547,8 +613,20 @@
       <c r="F6">
         <v>1.681</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>1.6652</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="1"/>
+        <v>1.6279999999999999</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="2"/>
+        <v>1.694</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -567,8 +645,20 @@
       <c r="F7">
         <v>9.3070000000000004</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>9.5366</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>9.2460000000000004</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="2"/>
+        <v>10.349</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -587,8 +677,20 @@
       <c r="F8">
         <v>49.643999999999998</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>53.140599999999992</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>49.218000000000004</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="2"/>
+        <v>67.064999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -607,8 +709,20 @@
       <c r="F9">
         <v>254.75399999999999</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>359.51400000000001</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>254.75399999999999</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="2"/>
+        <v>407.589</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -625,6 +739,18 @@
         <v>1255.2629999999999</v>
       </c>
       <c r="F10">
+        <v>1362.039</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>1254.1322</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="1"/>
+        <v>1203.059</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="2"/>
         <v>1362.039</v>
       </c>
     </row>

</xml_diff>